<commit_message>
lower RACP to 100
</commit_message>
<xml_diff>
--- a/InputData/elec/RACP/RPS Alternative Compliance Payment.xlsx
+++ b/InputData/elec/RACP/RPS Alternative Compliance Payment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28507"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\RACP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\elec\RACP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{BB0F855F-5615-4B6F-8C76-6AC2301E3C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDCC008A-FA0C-4FF5-B676-B8455495EAA1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9254CCF-C458-4F48-A572-2DA5437A4064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{987F1A2C-D0FF-46D7-8396-B08F06D764BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{987F1A2C-D0FF-46D7-8396-B08F06D764BF}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,9 +123,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -163,7 +163,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -269,7 +269,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -411,7 +411,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -420,19 +420,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FAF84CE-31BD-44F2-91E9-58D4BA5F9B1E}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -440,7 +440,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -456,19 +456,19 @@
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2">
-        <v>9999</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -482,14 +482,14 @@
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -503,15 +503,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -655,6 +646,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -662,13 +662,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EB15BFA-34E4-4DEF-AB2B-4231939C40D8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C8E66EB-CCF5-4195-811A-852CD62B6D3B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C8E66EB-CCF5-4195-811A-852CD62B6D3B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EB15BFA-34E4-4DEF-AB2B-4231939C40D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{511C0F96-ECA6-4DBB-A70D-43EC187AB105}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{511C0F96-ECA6-4DBB-A70D-43EC187AB105}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>